<commit_message>
test(metrics-utility): update report snapshots for opt-in defaults
Assisted-by: gpt-5.6-terra medium
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -9,10 +9,9 @@
   <sheets>
     <sheet name="Usage Reporting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Managed nodes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Indirectly Managed nodes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Usage by collections" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Usage by roles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Usage by modules" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Usage by collections" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Usage by roles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Usage by modules" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -915,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -930,18 +929,19 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Host name</t>
+          <t>Collection name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Automated by
-organizations</t>
+          <t>Unique managed nodes
+automated</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Job runs</t>
+          <t>Non-unique managed
+nodes automated</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
@@ -952,37 +952,8 @@
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>First
-automation</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t>Last
-automation</t>
-        </is>
-      </c>
-      <c r="G1" s="11" t="inlineStr">
-        <is>
-          <t>Canonical
-Facts</t>
-        </is>
-      </c>
-      <c r="H1" s="11" t="inlineStr">
-        <is>
-          <t>Facts</t>
-        </is>
-      </c>
-      <c r="I1" s="11" t="inlineStr">
-        <is>
-          <t>Manage
-Node
-Types</t>
-        </is>
-      </c>
-      <c r="J1" s="11" t="inlineStr">
-        <is>
-          <t>Events</t>
+          <t>Duration of task
+runs [seconds]</t>
         </is>
       </c>
     </row>
@@ -1012,7 +983,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Collection name</t>
+          <t>Role name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
@@ -1066,60 +1037,6 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Role name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
           <t>Module name</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Revert/aap 87148 metrics utility defaults (#579)
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -9,10 +9,9 @@
   <sheets>
     <sheet name="Usage Reporting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Managed nodes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Indirectly Managed nodes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Usage by collections" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Usage by roles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Usage by modules" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Usage by collections" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Usage by roles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Usage by modules" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -915,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -930,18 +929,19 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Host name</t>
+          <t>Collection name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Automated by
-organizations</t>
+          <t>Unique managed nodes
+automated</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Job runs</t>
+          <t>Non-unique managed
+nodes automated</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
@@ -952,37 +952,8 @@
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>First
-automation</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t>Last
-automation</t>
-        </is>
-      </c>
-      <c r="G1" s="11" t="inlineStr">
-        <is>
-          <t>Canonical
-Facts</t>
-        </is>
-      </c>
-      <c r="H1" s="11" t="inlineStr">
-        <is>
-          <t>Facts</t>
-        </is>
-      </c>
-      <c r="I1" s="11" t="inlineStr">
-        <is>
-          <t>Manage
-Node
-Types</t>
-        </is>
-      </c>
-      <c r="J1" s="11" t="inlineStr">
-        <is>
-          <t>Events</t>
+          <t>Duration of task
+runs [seconds]</t>
         </is>
       </c>
     </row>
@@ -1012,7 +983,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Collection name</t>
+          <t>Role name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
@@ -1066,60 +1037,6 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Role name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
           <t>Module name</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Revert "Revert/aap 87148 metrics utility defaults (#579)"
This reverts commit 67220f6b0a6bd13ed13f0caee44df7fc8ca2e02f.
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Usage Reporting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Managed nodes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Usage by collections" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Usage by roles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Usage by modules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Indirectly Managed nodes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Usage by collections" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Usage by roles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Usage by modules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -914,7 +915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -929,19 +930,18 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Collection name</t>
+          <t>Host name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Unique managed nodes
-automated</t>
+          <t>Automated by
+organizations</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Non-unique managed
-nodes automated</t>
+          <t>Job runs</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
@@ -952,8 +952,37 @@
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Duration of task
-runs [seconds]</t>
+          <t>First
+automation</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Last
+automation</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Canonical
+Facts</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Manage
+Node
+Types</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Events</t>
         </is>
       </c>
     </row>
@@ -983,7 +1012,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Role name</t>
+          <t>Collection name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
@@ -1037,6 +1066,60 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
+          <t>Role name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Unique managed nodes
+automated</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Non-unique managed
+nodes automated</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Number of task
+runs</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Duration of task
+runs [seconds]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
           <t>Module name</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Revert "Revert/aap 87148 metrics utility defaults (#579)" (#581)
This reverts commit 67220f6b0a6bd13ed13f0caee44df7fc8ca2e02f.
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Usage Reporting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Managed nodes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Usage by collections" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Usage by roles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Usage by modules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Indirectly Managed nodes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Usage by collections" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Usage by roles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Usage by modules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -914,7 +915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -929,19 +930,18 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Collection name</t>
+          <t>Host name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Unique managed nodes
-automated</t>
+          <t>Automated by
+organizations</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Non-unique managed
-nodes automated</t>
+          <t>Job runs</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
@@ -952,8 +952,37 @@
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Duration of task
-runs [seconds]</t>
+          <t>First
+automation</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Last
+automation</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Canonical
+Facts</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Manage
+Node
+Types</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Events</t>
         </is>
       </c>
     </row>
@@ -983,7 +1012,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Role name</t>
+          <t>Collection name</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
@@ -1037,6 +1066,60 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
+          <t>Role name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Unique managed nodes
+automated</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Non-unique managed
+nodes automated</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Number of task
+runs</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Duration of task
+runs [seconds]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
           <t>Module name</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Revert "[AAP-87150] Default-enable indirect node report sheets and report type in metrics-utility (ansible#559)"
This reverts commit 902ce04.
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -9,10 +9,6 @@
   <sheets>
     <sheet name="Usage Reporting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Managed nodes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Indirectly Managed nodes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Usage by collections" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Usage by roles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Usage by modules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -88,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0092d050"/>
+        <fgColor rgb="0000FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -907,248 +903,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Host name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Automated by
-organizations</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Job runs</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>First
-automation</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t>Last
-automation</t>
-        </is>
-      </c>
-      <c r="G1" s="11" t="inlineStr">
-        <is>
-          <t>Canonical
-Facts</t>
-        </is>
-      </c>
-      <c r="H1" s="11" t="inlineStr">
-        <is>
-          <t>Facts</t>
-        </is>
-      </c>
-      <c r="I1" s="11" t="inlineStr">
-        <is>
-          <t>Manage
-Node
-Types</t>
-        </is>
-      </c>
-      <c r="J1" s="11" t="inlineStr">
-        <is>
-          <t>Events</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Collection name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Role name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Module name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "[AAP-87150] Default-enable indirect node report sheets and report type in metrics-utility (ansible#559)" (#582)
This reverts commit 902ce04.
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -9,10 +9,6 @@
   <sheets>
     <sheet name="Usage Reporting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Managed nodes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Indirectly Managed nodes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Usage by collections" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Usage by roles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Usage by modules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -88,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0092d050"/>
+        <fgColor rgb="0000FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -907,248 +903,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Host name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Automated by
-organizations</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Job runs</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>First
-automation</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t>Last
-automation</t>
-        </is>
-      </c>
-      <c r="G1" s="11" t="inlineStr">
-        <is>
-          <t>Canonical
-Facts</t>
-        </is>
-      </c>
-      <c r="H1" s="11" t="inlineStr">
-        <is>
-          <t>Facts</t>
-        </is>
-      </c>
-      <c r="I1" s="11" t="inlineStr">
-        <is>
-          <t>Manage
-Node
-Types</t>
-        </is>
-      </c>
-      <c r="J1" s="11" t="inlineStr">
-        <is>
-          <t>Events</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Collection name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Role name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Module name</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Unique managed nodes
-automated</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Non-unique managed
-nodes automated</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Number of task
-runs</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Duration of task
-runs [seconds]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>